<commit_message>
GITBOOK-22: Fix typo file excel
</commit_message>
<xml_diff>
--- a/docs/0OMsoqOg9GiJ2xusVHMv/.gitbook/assets/IO - Template servizi - Multe per violazioni al Codice della Strada (1).xlsx
+++ b/docs/0OMsoqOg9GiJ2xusVHMv/.gitbook/assets/IO - Template servizi - Multe per violazioni al Codice della Strada (1).xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="75">
   <si>
     <r>
       <t xml:space="preserve">
@@ -437,8 +437,7 @@
         <sz val="10"/>
         <rFont val="Titillium Web"/>
       </rPr>
-      <t xml:space="preserve">
-[Vedi accertamento](URL)
+      <t xml:space="preserve"> - [Vedi accertamento](URL)
 </t>
     </r>
     <r>
@@ -500,7 +499,7 @@
         <sz val="10"/>
         <rFont val="Titillium Web"/>
       </rPr>
-      <t>&lt;gg/mm/aa&gt;</t>
+      <t>&lt;gg/mm/aaaa&gt;</t>
     </r>
     <r>
       <rPr>
@@ -509,8 +508,62 @@
         <rFont val="Titillium Web"/>
       </rPr>
       <t xml:space="preserve">? Riceverai il verbale di contravvenzione in base a quanto previsto dal Codice della Strada e potranno essere addebitate le spese di notifica. 
-Puoi pagare direttamente in app premendo “Vedi Avviso”, oppure tramite tutti i canali di pagamento della piattaforma pagoPA e le altre modalità di pagamento offerte dell'ente creditore.
-In fase di pagamento, se previsto dall'ente, l'importo riportato nel messaggio potrebbe subire variazioni.</t>
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="ff448844"/>
+        <family val="2"/>
+        <sz val="10"/>
+        <rFont val="Titillium Web"/>
+      </rPr>
+      <t>[Se previsto dal tipo di multa]</t>
+    </r>
+    <r>
+      <rPr>
+        <family val="2"/>
+        <sz val="10"/>
+        <rFont val="Titillium Web"/>
+      </rPr>
+      <t xml:space="preserve"> Inoltre, ricordati di [comunicare i dati di chi era alla guida del veicolo](URL) al momento dell'infrazione, anche se si tratta del proprietario del mezzo, entro il gg/mm/aaaa.
+Puoi pagare direttamente in app premendo “Paga”, oppure tramite tutti i canali di pagamento della piattaforma pagoPA e le altre modalità di pagamento offerte dell'ente creditore.
+In fase di pagamento, se previsto dall'ente, l'importo riportato nel messaggio potrebbe subire variazioni.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <family val="2"/>
+        <sz val="10"/>
+        <rFont val="Titillium Web"/>
+      </rPr>
+      <t>🪄  Pulsante 1:</t>
+    </r>
+    <r>
+      <rPr>
+        <family val="2"/>
+        <sz val="10"/>
+        <rFont val="Titillium Web"/>
+      </rPr>
+      <t xml:space="preserve"> Vedi accertamento
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <family val="2"/>
+        <sz val="10"/>
+        <rFont val="Titillium Web"/>
+      </rPr>
+      <t>🪄  Pulsante 2:</t>
+    </r>
+    <r>
+      <rPr>
+        <family val="2"/>
+        <sz val="10"/>
+        <rFont val="Titillium Web"/>
+      </rPr>
+      <t xml:space="preserve"> Paga (inserito automaticamente dall'app se il messaggio prevede un avviso di pagamento pagoPA)</t>
     </r>
   </si>
   <si>
@@ -553,9 +606,6 @@
       <t xml:space="preserve">
 Pulsante di azione primaria</t>
     </r>
-  </si>
-  <si>
-    <t>Vedi avviso</t>
   </si>
   <si>
     <t>-</t>
@@ -1265,12 +1315,12 @@
         <v>64</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="32" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B7" s="34" t="s">
         <v>52</v>
@@ -1281,43 +1331,43 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="34" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="32" t="s">
+      <c r="B9" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="C9" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="34" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="32" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="32" t="s">
+      <c r="B10" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="C10" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="C10" s="34" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="32" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="32" t="s">
+      <c r="B11" s="34" t="s">
         <v>74</v>
-      </c>
-      <c r="B11" s="34" t="s">
-        <v>75</v>
       </c>
       <c r="C11" s="34" t="s">
         <v>52</v>

</xml_diff>